<commit_message>
Refresh April code reader dashboard artifacts
</commit_message>
<xml_diff>
--- a/product_dashboard/data/code_reader_scanner/202604/summary.xlsx
+++ b/product_dashboard/data/code_reader_scanner/202604/summary.xlsx
@@ -12582,12 +12582,8 @@
       <c r="G8" t="n">
         <v>1055</v>
       </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B000EVYGV4</t>
@@ -12928,12 +12924,8 @@
       <c r="G20" t="n">
         <v>1055</v>
       </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B000EVYGV4</t>

</xml_diff>